<commit_message>
feat: add Colfert Power 12-61-0 product data
</commit_message>
<xml_diff>
--- a/wp-content/themes/eurofert-theme/scripts/products.xlsx
+++ b/wp-content/themes/eurofert-theme/scripts/products.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\eurofert\wp-content\themes\eurofert-theme\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E8ACE77-1E9F-49CA-B4B9-BFDDDCBF0837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E1A118-6303-4A73-966F-9F0F6EC97FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76D0BCB8-E73B-4392-8B84-A7325E8578D8}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
   <si>
     <t>title</t>
   </si>
@@ -125,6 +125,41 @@
   </si>
   <si>
     <t>K2O | 36.0 \n Organic Matter |50.0</t>
+  </si>
+  <si>
+    <t>Colfert Power 12-61-0</t>
+  </si>
+  <si>
+    <t>colfert-power</t>
+  </si>
+  <si>
+    <t>A unique formulation designed for root development and flowering stages, suitable for both fertigation and foliar spraying.
+Its high concentration of fully available phosphorus promotes the formation of a strong, dense root system, resulting in improved vegetative growth. It is also highly effective in rebuilding root systems following root diseases or nematode infections.
+When applied during the flowering stage, it helps stimulate flowering and increase flower numbers.
+Enriched with essential trace elements in balanced concentrations, it enhances plant strength and supports vigorous early growth.</t>
+  </si>
+  <si>
+    <t>High-Phosphorus Formula for Rooting &amp; Flowering</t>
+  </si>
+  <si>
+    <t>Chemically mixed, homogeneous NPK paste
+100% water-soluble and chloride-free
+Highly acidic – improves nutrient availability and system cleanliness
+Reduces algae growth and calcium deposits in drippers
+Compatible with most fertilizers and pesticides (compatibility test recommended)</t>
+  </si>
+  <si>
+    <t>12-61-0</t>
+  </si>
+  <si>
+    <t>Total Nitrogen | 12 
+Nitrate (NO3-N) | 0 
+Ammonium (NH4-N) |  12
+Urea (NH2-N) | 0
+Phosphate (P2O5) | 61 
+Potassium (K2O) | 0
+PH (1/1000) | 2.0 - 3.0
+Solubility g/lt at 20 C⁰ |  500</t>
   </si>
 </sst>
 </file>
@@ -992,7 +1027,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.44140625" customWidth="1"/>
     <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.109375" style="1" customWidth="1"/>
@@ -1104,7 +1139,7 @@
         <v>20</v>
       </c>
       <c r="B4" t="str">
-        <f t="shared" ref="B4:B5" si="0">SUBSTITUTE(LOWER(A4), " ", "-")</f>
+        <f t="shared" ref="B4:B6" si="0">SUBSTITUTE(LOWER(A4), " ", "-")</f>
         <v>colfert-essential-p</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -1114,7 +1149,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="1" t="str">
-        <f t="shared" ref="E4:E5" si="1">IF(B4="","", B4 &amp; ".webp")</f>
+        <f t="shared" ref="E4:E6" si="1">IF(B4="","", B4 &amp; ".webp")</f>
         <v>colfert-essential-p.webp</v>
       </c>
       <c r="F4" t="s">
@@ -1158,6 +1193,41 @@
       <c r="J5" s="1" t="str">
         <f>IF(B5="","", B5 &amp; ".json")</f>
         <v>colfert-essential-pk.json</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="288" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="str">
+        <f>SUBSTITUTE(LOWER(A6), " ", "-")</f>
+        <v>colfert-power-12-61-0</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>colfert-power-12-61-0.webp</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J6" s="1" t="str">
+        <f>IF(B6="","", B6 &amp; ".json")</f>
+        <v>colfert-power-12-61-0.json</v>
       </c>
     </row>
     <row r="22" spans="4:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Redesign product details page and optimize recommendation table UI
</commit_message>
<xml_diff>
--- a/wp-content/themes/eurofert-theme/scripts/products.xlsx
+++ b/wp-content/themes/eurofert-theme/scripts/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\eurofert\wp-content\themes\eurofert-theme\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E1A118-6303-4A73-966F-9F0F6EC97FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECAFD889-E504-40E7-AF51-FB750AC88BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76D0BCB8-E73B-4392-8B84-A7325E8578D8}"/>
   </bookViews>
@@ -149,9 +149,6 @@
 Compatible with most fertilizers and pesticides (compatibility test recommended)</t>
   </si>
   <si>
-    <t>12-61-0</t>
-  </si>
-  <si>
     <t>Total Nitrogen | 12 
 Nitrate (NO3-N) | 0 
 Ammonium (NH4-N) |  12
@@ -160,6 +157,9 @@
 Potassium (K2O) | 0
 PH (1/1000) | 2.0 - 3.0
 Solubility g/lt at 20 C⁰ |  500</t>
+  </si>
+  <si>
+    <t>12-61-0+TE</t>
   </si>
 </sst>
 </file>
@@ -1026,7 +1026,7 @@
   <dimension ref="A1:J30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.44140625" customWidth="1"/>
     <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
@@ -1139,7 +1139,7 @@
         <v>20</v>
       </c>
       <c r="B4" t="str">
-        <f t="shared" ref="B4:B6" si="0">SUBSTITUTE(LOWER(A4), " ", "-")</f>
+        <f t="shared" ref="B4:B5" si="0">SUBSTITUTE(LOWER(A4), " ", "-")</f>
         <v>colfert-essential-p</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -1220,10 +1220,10 @@
         <v>34</v>
       </c>
       <c r="H6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="J6" s="1" t="str">
         <f>IF(B6="","", B6 &amp; ".json")</f>

</xml_diff>

<commit_message>
feat: add Colfert Power 15-20-50, 20-20-20, and 20-50-10 datasheets and update products.xlsx
</commit_message>
<xml_diff>
--- a/wp-content/themes/eurofert-theme/scripts/products.xlsx
+++ b/wp-content/themes/eurofert-theme/scripts/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\eurofert\wp-content\themes\eurofert-theme\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECAFD889-E504-40E7-AF51-FB750AC88BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF425181-466E-457F-91B3-294C70C4DF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76D0BCB8-E73B-4392-8B84-A7325E8578D8}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="50">
   <si>
     <t>title</t>
   </si>
@@ -160,6 +160,69 @@
   </si>
   <si>
     <t>12-61-0+TE</t>
+  </si>
+  <si>
+    <t>High-Potassium Formula for Fruiting &amp; Ripening</t>
+  </si>
+  <si>
+    <t>Colfert Power 15-20-50</t>
+  </si>
+  <si>
+    <t>A specialized formulation designed to enhance fruit size, quality, and yield.
+Its high potassium content increases the sugar and carbohydrate levels in fruits, improving taste and market value.
+Recommended for use during the fruiting and ripening stages to maintain an optimal balance between vegetative growth and fruit development, extending the crop’s productive life.
+Enriched with essential micronutrients to ensure healthy growth and prevent deficiencies.</t>
+  </si>
+  <si>
+    <t>15-20-50 +TE</t>
+  </si>
+  <si>
+    <t>Total Nitrogen|15
+Nitrate (NO3-N)|8
+Ammonium (NH4-N)|4
+Urea (NH2-N)|3
+Phosphate (P2O5)|20
+Potassium (K2O)|50
+pH (1/1000)|2.0 - 3.0
+Solubility g/lt at 20 C°|250</t>
+  </si>
+  <si>
+    <t>Colfert Power 20-20-20</t>
+  </si>
+  <si>
+    <t>Balanced NPK Formula</t>
+  </si>
+  <si>
+    <t>A balanced formulation that serves as a general-purpose fertilizer suitable for all crops designed to correct deficiencies in major nutrients.
+Ideal for crops with gradual ripening, requiring simultaneous high levels of N, P, and K to support new flower development, fruit ripening, and vegetative growth.
+Thanks to its unique chemical structure, this formula offers higher efficiency than conventional balanced NPK products.
+Enriched with essential micronutrients to promote healthy plant growth and prevent nutrient deficiencies.</t>
+  </si>
+  <si>
+    <t>20-20-20 +TE</t>
+  </si>
+  <si>
+    <t>Total Nitrogen|20
+Nitrate (NO3-N)|5.5
+Ammonium (NH4-N)|9
+Urea (NH2-N)|5.5
+Phosphate (P2O5)|20
+Potassium (K2O)|20
+pH (1/1000)|2.0 - 3.0
+Solubility g/lt at 20 C°|300</t>
+  </si>
+  <si>
+    <t>Colfert Power 20-50-10</t>
+  </si>
+  <si>
+    <t>Colfert Power 20-50-10+TE</t>
+  </si>
+  <si>
+    <t>A unique formulation designed for the root development and flowering stages, suitable for both fertigation and foliar application.
+The high concentration of fully available phosphorus promotes a strong, dense root system, leading to better vegetative growth.
+Adequate levels of potassium enhance disease resistance and tolerance to adverse conditions, while also helping restore root systems affected by root diseases or nematode damage.
+When applied during the flowering stage, it stimulates flower initiation and increases flower numbers.
+Enriched with balanced trace elements, it strengthens the plant and supports vigorous early growth.</t>
   </si>
 </sst>
 </file>
@@ -1027,13 +1090,13 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.44140625" customWidth="1"/>
     <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="41.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="32.77734375" customWidth="1"/>
-    <col min="8" max="8" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" customWidth="1"/>
     <col min="9" max="9" width="18.5546875" customWidth="1"/>
     <col min="10" max="10" width="26.21875" style="1" customWidth="1"/>
   </cols>
@@ -1149,7 +1212,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="1" t="str">
-        <f t="shared" ref="E4:E6" si="1">IF(B4="","", B4 &amp; ".webp")</f>
+        <f t="shared" ref="E4:E9" si="1">IF(B4="","", B4 &amp; ".webp")</f>
         <v>colfert-essential-p.webp</v>
       </c>
       <c r="F4" t="s">
@@ -1228,6 +1291,108 @@
       <c r="J6" s="1" t="str">
         <f>IF(B6="","", B6 &amp; ".json")</f>
         <v>colfert-power-12-61-0.json</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="str">
+        <f>SUBSTITUTE(LOWER(A7), " ", "-")</f>
+        <v>colfert-power-15-20-50</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>colfert-power-15-20-50.webp</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H7" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J7" s="1" t="str">
+        <f>IF(B7="","", B7 &amp; ".json")</f>
+        <v>colfert-power-15-20-50.json</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" t="str">
+        <f>SUBSTITUTE(LOWER(A8), " ", "-")</f>
+        <v>colfert-power-20-20-20</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>colfert-power-20-20-20.webp</v>
+      </c>
+      <c r="F8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>45</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J8" s="1" t="str">
+        <f>IF(B8="","", B8 &amp; ".json")</f>
+        <v>colfert-power-20-20-20.json</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="288" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="str">
+        <f>SUBSTITUTE(LOWER(A9), " ", "-")</f>
+        <v>colfert-power-20-50-10</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>colfert-power-20-50-10.webp</v>
+      </c>
+      <c r="F9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" s="1" t="str">
+        <f>IF(B9="","", B9 &amp; ".json")</f>
+        <v>colfert-power-20-50-10.json</v>
       </c>
     </row>
     <row r="22" spans="4:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
chore: update products datasheet and local sync metadata
</commit_message>
<xml_diff>
--- a/wp-content/themes/eurofert-theme/scripts/products.xlsx
+++ b/wp-content/themes/eurofert-theme/scripts/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\eurofert\wp-content\themes\eurofert-theme\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF425181-466E-457F-91B3-294C70C4DF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C392C55-2348-4507-B5A2-4F3A5F4BD804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76D0BCB8-E73B-4392-8B84-A7325E8578D8}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="51">
   <si>
     <t>title</t>
   </si>
@@ -223,6 +223,9 @@
 Adequate levels of potassium enhance disease resistance and tolerance to adverse conditions, while also helping restore root systems affected by root diseases or nematode damage.
 When applied during the flowering stage, it stimulates flower initiation and increases flower numbers.
 Enriched with balanced trace elements, it strengthens the plant and supports vigorous early growth.</t>
+  </si>
+  <si>
+    <t>Total Nitrogen|20\nNitrate (NO3-N)|0\nAmmonium (NH4-N)|2\nUrea (NH2-N)|18\nPhosphate (P2O5)|50\nPotassium (K2O)|10\npH (1/1000)|2.5 - 3.5\nSolubility g/lt at 20 C°|400</t>
   </si>
 </sst>
 </file>
@@ -1390,6 +1393,9 @@
       <c r="H9" t="s">
         <v>48</v>
       </c>
+      <c r="I9" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="J9" s="1" t="str">
         <f>IF(B9="","", B9 &amp; ".json")</f>
         <v>colfert-power-20-50-10.json</v>

</xml_diff>

<commit_message>
added all foliar products
</commit_message>
<xml_diff>
--- a/wp-content/themes/eurofert-theme/scripts/products.xlsx
+++ b/wp-content/themes/eurofert-theme/scripts/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\eurofert\wp-content\themes\eurofert-theme\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2231BCE5-4B78-4776-819B-B41D5A426B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1094B55-5BAA-45DA-9926-8288F1356D8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,8 +32,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="67">
   <si>
     <t>title</t>
   </si>
@@ -93,9 +115,6 @@
   </si>
   <si>
     <t>Enhances fruit size, sugar content, and color development\n Improves soil properties, buffering capacity, and microbial activity.\nIncreases plant vitality, vigor, and disease resistance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0-0-36+ 50% </t>
   </si>
   <si>
     <t>K2O | 36.0 \n Organic Matter |50.0</t>
@@ -147,9 +166,6 @@
 Highly acidic – improves nutrient availability and system cleanliness_x000D_
 Reduces algae growth and calcium deposits in drippers_x000D_
 Compatible with most fertilizers and pesticides (compatibility test recommended)</t>
-  </si>
-  <si>
-    <t>12-61-0+TE</t>
   </si>
   <si>
     <t>Total Nitrogen | 12 _x000D_
@@ -174,19 +190,6 @@
     <t>High-Potassium Formula for Fruiting &amp; Ripening</t>
   </si>
   <si>
-    <t>15-20-50 +TE</t>
-  </si>
-  <si>
-    <t>Total Nitrogen|15_x000D_
-Nitrate (NO3-N)|8_x000D_
-Ammonium (NH4-N)|4_x000D_
-Urea (NH2-N)|3_x000D_
-Phosphate (P2O5)|20_x000D_
-Potassium (K2O)|50_x000D_
-pH (1/1000)|2.0 - 3.0_x000D_
-Solubility g/lt at 20 C°|250</t>
-  </si>
-  <si>
     <t>Colfert Power 20-20-20</t>
   </si>
   <si>
@@ -197,9 +200,6 @@
   </si>
   <si>
     <t>Balanced NPK Formula</t>
-  </si>
-  <si>
-    <t>20-20-20 +TE</t>
   </si>
   <si>
     <t>Total Nitrogen|20_x000D_
@@ -225,9 +225,6 @@
     <t>Total Nitrogen|20\nNitrate (NO3-N)|0\nAmmonium (NH4-N)|2\nUrea (NH2-N)|18\nPhosphate (P2O5)|50\nPotassium (K2O)|10\npH (1/1000)|2.5 - 3.5\nSolubility g/lt at 20 C°|400</t>
   </si>
   <si>
-    <t>Colfert Foliar 30-10-10+TE</t>
-  </si>
-  <si>
     <t>The Colfert foliar NPK fertilizer range is formulated to deliver essential nutrients directly through the leaves for fast, efficient absorption. This advanced formulation promotes vigorous vegetative growth, enhances flowering and fruit set, and significantly improves both yield and quality.</t>
   </si>
   <si>
@@ -247,16 +244,119 @@
 Compatible with most fertilizers and pesticides (compatibility test recommended)</t>
   </si>
   <si>
-    <t>20-50-10+TE</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 30-10-10+TE</t>
-  </si>
-  <si>
     <t>High N</t>
   </si>
   <si>
     <t>Total Nitrogen | 30 \n Ammoniacal-N (NH4-N) | 2 \n Nitric-N (NO3-N) | 2.9 \n Ureic-N (NH2-N) | 25.1 \n Phosphate (P2O5) | 10 \n Potassium (K2O) | 10 \n Magnesium (MgO) | 2 \n Sulfur Trioxide (SO3) | 4 \n Boron | 0.01 \n Copper* | 0.02 \n Iron* | 0.05 \n Manganese* | 0.04 \n Molybdenum | 0.001 \n Zinc* | 0.02</t>
+  </si>
+  <si>
+    <t>recommendations_json</t>
+  </si>
+  <si>
+    <t>[{"crop":"Arable crops, vegetables, fruit trees","fertigation":"2 – 5 Kg/Ha","foliar":"","time":""},{"crop":"Nurseries &amp; Ornamentals","fertigation":"150 – 300 g/100 L of water","foliar":"","time":""}]</t>
+  </si>
+  <si>
+    <t>1 kg, 10 kg, 25kg</t>
+  </si>
+  <si>
+    <t>Colfert Foliar 30-10-10 +TE</t>
+  </si>
+  <si>
+    <t>Colfert Foliar 10-10-40 +TE</t>
+  </si>
+  <si>
+    <t>High K</t>
+  </si>
+  <si>
+    <t>0-0-36+ 50%</t>
+  </si>
+  <si>
+    <t>Total Nitrogen|15
+Nitrate (NO3-N)|8
+Ammonium (NH4-N)|4
+Urea (NH2-N)|3
+Phosphate (P2O5)|20
+Potassium (K2O)|50
+pH (1/1000)|2.0 - 3.0
+Solubility g/lt at 20 C°|250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Nitrogen|10
+Ammoniacal-N (NH4-N)|0
+Nitric-N (NO3-N)|5.4
+Ureic-N (NH2-N)|4.6
+Phosphate (P2O5)|10
+Potassium (K2O)|40
+Sulfur Trioxide (SO3)|13.5
+Boron|0.01
+Copper*|0.02
+Iron*|0.05
+Manganese*|0.04
+Molybdenum|0.001
+Zinc*|0.02 </t>
+  </si>
+  <si>
+    <t>Colfert Foliar 20-20-20 +TE</t>
+  </si>
+  <si>
+    <t>Balance</t>
+  </si>
+  <si>
+    <t>Total Nitrogen|20
+Ammoniacal-N (NH4-N)|2.4
+Nitric-N (NO3-N)|4.3
+Ureic-N (NH2-N)|13.2
+Phosphate (P2O5)|20
+Potassium (K2O)|20
+Magnesium (MgO)|1
+Sulfur Trioxide (SO3)|2
+Boron|0.01
+Copper*|0.02
+Iron*|0.05
+Manganese*|0.04
+Molybdenum|0.001
+Zinc*|0.02</t>
+  </si>
+  <si>
+    <t>Colfert Foliar 12-48-8 +TE</t>
+  </si>
+  <si>
+    <t>High P</t>
+  </si>
+  <si>
+    <t>Total Nitrogen|12
+Ammoniacal-N (NH4-N)|8
+Nitric-N (NO3-N)|0
+Ureic-N (NH2-N)|4
+Phosphate (P2O5)|48
+Potassium (K2O)|8
+Magnesium (MgO)|1
+Sulfur Trioxide (SO3)|5
+Boron|0.01
+Copper*|0.02
+Iron*|0.05
+Manganese*|0.04
+Molybdenum|0.001
+Zinc*|0.02</t>
+  </si>
+  <si>
+    <t>Colfert Foliar 15-5-30 +TE</t>
+  </si>
+  <si>
+    <t>Total Nitrogen|15
+Ammoniacal-N (NH4-N)|1
+Nitric-N (NO3-N)|3.7
+Ureic-N (NH2-N)|10.3
+Phosphate (P2O5)|5
+Potassium (K2O)|30
+Magnesium (MgO)|2
+Sulfur Trioxide (SO3)|19.5
+Boron|0.01
+Copper*|0.02
+Iron*|0.05
+Manganese*|0.04
+Molybdenum|0.001
+Zinc*|0.02</t>
   </si>
 </sst>
 </file>
@@ -292,14 +392,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -310,6 +417,40 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0494B0DF-D027-438F-A4D2-293CE04AC4BE}" name="Table1" displayName="Table1" ref="A1:L18" totalsRowShown="0">
+  <autoFilter ref="A1:L18" xr:uid="{0494B0DF-D027-438F-A4D2-293CE04AC4BE}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{5D4C21B3-8D7F-41A5-AC7F-965FB9BE6891}" name="title"/>
+    <tableColumn id="2" xr3:uid="{26889905-EFE8-44C5-AE7C-032F4B9915DB}" name="slug"/>
+    <tableColumn id="3" xr3:uid="{1B8C8307-7500-428E-870A-CD033ADFD8F3}" name="content"/>
+    <tableColumn id="4" xr3:uid="{BF5C3923-6BEF-4A4E-974F-953FB204BE94}" name="category_slug"/>
+    <tableColumn id="5" xr3:uid="{ACED1FE6-92D4-4BC5-A6F9-DBC13553C30E}" name="local_image_path">
+      <calculatedColumnFormula>IF(B2="", "", B2 &amp; ".webp")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{F54B9109-FAE1-460E-8C88-87A5D7AC75BB}" name="subtitle"/>
+    <tableColumn id="7" xr3:uid="{0FC1B192-DEF0-4CED-86DB-754595426F1E}" name="key_benefits" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{EB479CD4-CE24-41F9-BFBC-1E024C798CF6}" name="formula">
+      <calculatedColumnFormula array="1">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{7C10BDA6-8F0D-40B4-9479-697DDBDC92FF}" name="nutrient_rows"/>
+    <tableColumn id="10" xr3:uid="{C688EF8B-08F1-4BD7-97DD-31658417BA5A}" name="recommendations_file_path">
+      <calculatedColumnFormula>IF(L2&lt;&gt;"", "", IF(B2="", "", B2 &amp; ".json"))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{D9E2066C-B7AA-4003-9F8B-834D537C71A6}" name="packages_content"/>
+    <tableColumn id="12" xr3:uid="{4175EFED-3B8F-4F2E-AB1F-DF3A7543149D}" name="recommendations_json"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -629,22 +770,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.69921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.296875" customWidth="1"/>
     <col min="3" max="3" width="9.19921875" customWidth="1"/>
     <col min="4" max="4" width="14.19921875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.59765625" customWidth="1"/>
-    <col min="7" max="7" width="10.69921875" customWidth="1"/>
+    <col min="6" max="6" width="8.8984375" customWidth="1"/>
+    <col min="7" max="7" width="26.8984375" style="2" customWidth="1"/>
     <col min="8" max="8" width="11.3984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.3984375" customWidth="1"/>
-    <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="15.5" customWidth="1"/>
+    <col min="9" max="9" width="14.09765625" customWidth="1"/>
+    <col min="10" max="10" width="25.796875" customWidth="1"/>
+    <col min="11" max="11" width="17.69921875" customWidth="1"/>
+    <col min="12" max="12" width="22.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -663,7 +806,7 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="H1" t="s">
@@ -678,8 +821,11 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -701,7 +847,7 @@
       <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H2" t="s">
@@ -715,33 +861,33 @@
         <v>colfert-essential-n.json</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
       <c r="B3" t="str">
-        <f t="shared" ref="B3:B14" si="0">LOWER(SUBSTITUTE(SUBSTITUTE(TRIM(A3), "+TE", ""), " ", "-"))</f>
+        <f t="shared" ref="B3:B9" si="0">LOWER(SUBSTITUTE(SUBSTITUTE(TRIM(A3), "+TE", ""), " ", "-"))</f>
         <v>colfert-essential-ktc</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
       </c>
       <c r="D3" t="str">
-        <f t="shared" ref="D3:D18" si="1">IFERROR(LEFT(B3, FIND("-", B3, FIND("-", B3) + 1) - 1), B3)</f>
+        <f t="shared" ref="D3:D17" si="1">IFERROR(LEFT(B3, FIND("-", B3, FIND("-", B3) + 1) - 1), B3)</f>
         <v>colfert-essential</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" ref="E3:E18" si="2">IF(B3="", "", B3 &amp; ".webp")</f>
         <v>colfert-essential-ktc.webp</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I3" t="s">
         <v>20</v>
-      </c>
-      <c r="I3" t="s">
-        <v>21</v>
       </c>
       <c r="J3" t="str">
         <f t="shared" ref="J3:J18" si="3">IF(B3="", "", B3 &amp; ".json")</f>
@@ -751,16 +897,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>colfert-essential-p</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" si="1"/>
@@ -771,16 +917,13 @@
         <v>colfert-essential-p.webp</v>
       </c>
       <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" t="s">
         <v>24</v>
       </c>
-      <c r="G4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>25</v>
-      </c>
-      <c r="I4" t="s">
-        <v>26</v>
       </c>
       <c r="J4" t="str">
         <f t="shared" si="3"/>
@@ -790,16 +933,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>colfert-essential-pk</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="1"/>
@@ -812,14 +955,11 @@
       <c r="F5" t="s">
         <v>13</v>
       </c>
-      <c r="G5" t="s">
-        <v>13</v>
-      </c>
       <c r="H5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
         <v>29</v>
-      </c>
-      <c r="I5" t="s">
-        <v>30</v>
       </c>
       <c r="J5" t="str">
         <f t="shared" si="3"/>
@@ -829,16 +969,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>colfert-power-12-61-0</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="1"/>
@@ -849,16 +989,24 @@
         <v>colfert-power-12-61-0.webp</v>
       </c>
       <c r="F6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="str" cm="1">
+        <f t="array" ref="H6">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v>12-61-0</v>
+      </c>
+      <c r="I6" t="s">
         <v>34</v>
-      </c>
-      <c r="H6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I6" t="s">
-        <v>36</v>
       </c>
       <c r="J6" t="str">
         <f t="shared" si="3"/>
@@ -868,16 +1016,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="16.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>colfert-power-15-20-50</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="1"/>
@@ -888,16 +1036,24 @@
         <v>colfert-power-15-20-50.webp</v>
       </c>
       <c r="F7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" t="s">
-        <v>34</v>
-      </c>
-      <c r="H7" t="s">
-        <v>40</v>
-      </c>
-      <c r="I7" t="s">
-        <v>41</v>
+        <v>37</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="str" cm="1">
+        <f t="array" ref="H7">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v>15-20-50</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>57</v>
       </c>
       <c r="J7" t="str">
         <f t="shared" si="3"/>
@@ -907,16 +1063,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>colfert-power-20-20-20</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="1"/>
@@ -927,16 +1083,24 @@
         <v>colfert-power-20-20-20.webp</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G8" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" t="s">
-        <v>45</v>
+        <v>40</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" t="str" cm="1">
+        <f t="array" ref="H8">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v>20-20-20</v>
       </c>
       <c r="I8" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="J8" t="str">
         <f t="shared" si="3"/>
@@ -946,16 +1110,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>colfert-power-20-50-10</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="1"/>
@@ -966,16 +1130,24 @@
         <v>colfert-power-20-50-10.webp</v>
       </c>
       <c r="F9" t="s">
-        <v>33</v>
-      </c>
-      <c r="G9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H9" t="s">
-        <v>54</v>
+        <v>32</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" t="str" cm="1">
+        <f t="array" ref="H9">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v>20-50-10</v>
       </c>
       <c r="I9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="J9" t="str">
         <f t="shared" si="3"/>
@@ -985,16 +1157,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B10" t="str">
-        <f>LOWER(SUBSTITUTE(SUBSTITUTE(TRIM(A10), "+TE", ""), " ", "-"))</f>
+        <f>LOWER(SUBSTITUTE(TRIM(SUBSTITUTE(A10, "+TE", "")), " ", "-"))</f>
         <v>colfert-foliar-30-10-10</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="1"/>
@@ -1005,179 +1177,237 @@
         <v>colfert-foliar-30-10-10.webp</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G10" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" t="str" cm="1">
+        <f t="array" ref="H10">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v>30-10-10</v>
+      </c>
+      <c r="I10" t="s">
+        <v>49</v>
+      </c>
+      <c r="J10" t="str">
+        <f>IF(L10&lt;&gt;"", "", IF(B10="", "", B10 &amp; ".json"))</f>
+        <v/>
+      </c>
+      <c r="K10" t="s">
         <v>52</v>
       </c>
-      <c r="H10" t="s">
-        <v>55</v>
-      </c>
-      <c r="I10" t="s">
-        <v>57</v>
-      </c>
-      <c r="J10" t="str">
-        <f t="shared" si="3"/>
-        <v>colfert-foliar-30-10-10.json</v>
-      </c>
-      <c r="K10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
       <c r="B11" t="str">
-        <f t="shared" ref="B11:B14" si="4">LOWER(SUBSTITUTE(SUBSTITUTE(TRIM(A11), "+TE", ""), " ", "-"))</f>
-        <v/>
+        <f t="shared" ref="B11:B14" si="4">LOWER(SUBSTITUTE(TRIM(SUBSTITUTE(A11, "+TE", "")), " ", "-"))</f>
+        <v>colfert-foliar-10-10-40</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>colfert-foliar</v>
       </c>
       <c r="E11" t="str">
         <f>IF(B11="", "", B11 &amp; ".webp")</f>
-        <v/>
+        <v>colfert-foliar-10-10-40.webp</v>
       </c>
       <c r="F11" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H11" t="s">
-        <v>13</v>
-      </c>
-      <c r="I11" t="s">
-        <v>13</v>
+        <v>55</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" t="str" cm="1">
+        <f t="array" ref="H11">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v>10-10-40</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>58</v>
       </c>
       <c r="J11" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="J11:J18" si="5">IF(L11&lt;&gt;"", "", IF(B11="", "", B11 &amp; ".json"))</f>
         <v/>
       </c>
       <c r="K11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+      <c r="L11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>colfert-foliar-20-20-20</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>colfert-foliar</v>
       </c>
       <c r="E12" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>colfert-foliar-20-20-20.webp</v>
       </c>
       <c r="F12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I12" t="s">
-        <v>13</v>
+        <v>60</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H12" t="str" cm="1">
+        <f t="array" ref="H12">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v>20-20-20</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>61</v>
       </c>
       <c r="J12" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+      <c r="L12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>colfert-foliar-12-48-8</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="D13" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>colfert-foliar</v>
       </c>
       <c r="E13" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>colfert-foliar-12-48-8.webp</v>
       </c>
       <c r="F13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I13" t="s">
-        <v>13</v>
+        <v>63</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H13" t="str" cm="1">
+        <f t="array" ref="H13">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v>12-48-8</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>64</v>
       </c>
       <c r="J13" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+      <c r="L13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>colfert-foliar-15-5-30</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="D14" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>colfert-foliar</v>
       </c>
       <c r="E14" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>colfert-foliar-15-5-30.webp</v>
       </c>
       <c r="F14" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14" t="s">
-        <v>13</v>
-      </c>
-      <c r="I14" t="s">
-        <v>13</v>
+        <v>55</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H14" t="str" cm="1">
+        <f t="array" ref="H14">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v>15-5-30</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="J14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+      <c r="L14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1191,24 +1421,29 @@
       <c r="F15" t="s">
         <v>13</v>
       </c>
-      <c r="G15" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" t="s">
-        <v>13</v>
+      <c r="H15" t="str" cm="1">
+        <f t="array" ref="H15">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v/>
       </c>
       <c r="I15" t="s">
         <v>13</v>
       </c>
       <c r="J15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1229,17 +1464,22 @@
       <c r="F16" t="s">
         <v>13</v>
       </c>
-      <c r="G16" t="s">
-        <v>13</v>
-      </c>
-      <c r="H16" t="s">
-        <v>13</v>
+      <c r="H16" t="str" cm="1">
+        <f t="array" ref="H16">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v/>
       </c>
       <c r="I16" t="s">
         <v>13</v>
       </c>
       <c r="J16" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K16" t="s">
@@ -1267,17 +1507,22 @@
       <c r="F17" t="s">
         <v>13</v>
       </c>
-      <c r="G17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" t="s">
-        <v>13</v>
+      <c r="H17" t="str" cm="1">
+        <f t="array" ref="H17">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v/>
       </c>
       <c r="I17" t="s">
         <v>13</v>
       </c>
       <c r="J17" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K17" t="s">
@@ -1298,17 +1543,22 @@
       <c r="F18" t="s">
         <v>13</v>
       </c>
-      <c r="G18" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" t="s">
-        <v>13</v>
+      <c r="H18" t="str" cm="1">
+        <f t="array" ref="H18">IF(COUNT(FIND({0,1,2,3,4,5,6,7,8,9}, Table1[[#This Row],[title]]))=0, "",
+    _xlfn.LET(
+        _xlpm.text, Table1[[#This Row],[title]],
+        _xlpm.startNum, MIN(FIND({0,1,2,3,4,5,6,7,8,9}, _xlpm.text&amp;"0123456789")),
+        _xlpm.endSpace, FIND(" ", _xlpm.text&amp;" ", _xlpm.startNum),
+        MID(_xlpm.text, _xlpm.startNum, _xlpm.endSpace - _xlpm.startNum)
+    )
+)</f>
+        <v/>
       </c>
       <c r="I18" t="s">
         <v>13</v>
       </c>
       <c r="J18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K18" t="s">
@@ -1317,8 +1567,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A4:A5 A1:C1 A12:A14 C9 A3 C3 A7:A8 A6 C6 I9 F2:G2 G3 K10 C11 C4:C5 C7:C8 F1:I1 A18 C18 A16:C17 A15 C15 F6:I6 F5:G5 F7:I8 K9 K3 K6 K4:K5 K7:K8 C12:C14 F11:I11 F18:I18 F16:I17 F15:I15 F12:I14 K11 K18 K16:K17 K15 K12:K14 I3 F4:G4 I4 I5" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>